<commit_message>
Fix: Updated Excel tab name to match AddTickers test method
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Archana\eclipse-workspace\delta1-automation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14E0A6EF-6ECA-4203-B58B-04EC01C07160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D74CDE-0F31-433C-B311-D89CF5B1FF92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" firstSheet="1" activeTab="1" xr2:uid="{5F4CC7F0-8BD6-41FD-85C1-DCF17C64A46A}"/>
   </bookViews>
@@ -1061,80 +1061,80 @@
   <volType type="realTimeData">
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...3689127776</v>
+        <v>#N/A Requesting Data...3116730286</v>
         <stp/>
         <stp>BDP|14014614177385490883</stp>
         <tr r="M11" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3627122317</v>
+        <v>#N/A Requesting Data...3323881689</v>
         <stp/>
         <stp>BDP|17914771070757396967</stp>
         <tr r="M23" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4116552338</v>
+        <v>#N/A Requesting Data...1831997750</v>
         <stp/>
         <stp>BDP|12191885856176020024</stp>
         <tr r="M19" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3756918296</v>
+        <v>#N/A Requesting Data...3539005372</v>
         <stp/>
         <stp>BDP|11222918239606141336</stp>
         <tr r="M10" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4015068224</v>
+        <v>#N/A Requesting Data...1921182470</v>
         <stp/>
         <stp>BDP|10651803860804892507</stp>
         <tr r="M20" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3855679841</v>
+        <v>#N/A Requesting Data...2863434980</v>
         <stp/>
         <stp>BDP|11138132499892845425</stp>
         <tr r="B6" s="4"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3336474272</v>
+        <v>#N/A Requesting Data...2809252556</v>
         <stp/>
         <stp>BDP|14818210720281309974</stp>
         <tr r="F4" s="4"/>
         <tr r="M24" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3772893482</v>
+        <v>#N/A Requesting Data...3915597306</v>
         <stp/>
         <stp>BDP|17354182839553220513</stp>
         <tr r="M18" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3528778928</v>
+        <v>#N/A Requesting Data...2702786370</v>
         <stp/>
         <stp>BDP|15833637773500916777</stp>
         <tr r="M22" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4150091446</v>
+        <v>#N/A Requesting Data...3858587456</v>
         <stp/>
         <stp>BDP|10553485173797766561</stp>
         <tr r="M17" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3213968450</v>
+        <v>#N/A Requesting Data...2028483817</v>
         <stp/>
         <stp>BDP|10725320790729783234</stp>
         <tr r="M8" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4151063015</v>
+        <v>#N/A Requesting Data...2905634664</v>
         <stp/>
         <stp>BDP|15290075098549931204</stp>
         <tr r="M2" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4283927025</v>
+        <v>#N/A Requesting Data...1818396705</v>
         <stp/>
         <stp>BDP|11090127615376453378</stp>
         <tr r="M13" s="5"/>
@@ -1142,19 +1142,19 @@
     </main>
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...3405367639</v>
+        <v>#N/A Requesting Data...2463032671</v>
         <stp/>
         <stp>BDP|4236539151683226891</stp>
         <tr r="M21" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3322533595</v>
+        <v>#N/A Requesting Data...3415227157</v>
         <stp/>
         <stp>BDP|2613081399981359290</stp>
         <tr r="M12" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3382180936</v>
+        <v>#N/A Requesting Data...2945205562</v>
         <stp/>
         <stp>BDP|2154512199383777756</stp>
         <tr r="M6" s="5"/>
@@ -1172,7 +1172,7 @@
         <tr r="N23" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3464180546</v>
+        <v>#N/A Requesting Data...4254932893</v>
         <stp/>
         <stp>BDP|2219595241806083194</stp>
         <tr r="M15" s="5"/>
@@ -1185,37 +1185,37 @@
         <tr r="E16" s="4"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3490270653</v>
+        <v>#N/A Requesting Data...3813285549</v>
         <stp/>
         <stp>BDP|7276645360862777315</stp>
         <tr r="M5" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4026368147</v>
+        <v>#N/A Requesting Data...3271659411</v>
         <stp/>
         <stp>BDP|1614643148556376256</stp>
         <tr r="M9" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3471357210</v>
+        <v>#N/A Requesting Data...3800748930</v>
         <stp/>
         <stp>BDP|8389300253224362856</stp>
         <tr r="M4" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3739426020</v>
+        <v>#N/A Requesting Data...3710702205</v>
         <stp/>
         <stp>BDP|1386483162619383929</stp>
         <tr r="M3" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4184503431</v>
+        <v>#N/A Requesting Data...2644152884</v>
         <stp/>
         <stp>BDP|722161999546011081</stp>
         <tr r="M14" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3861328267</v>
+        <v>#N/A Requesting Data...2559657153</v>
         <stp/>
         <stp>BDP|281963796682346956</stp>
         <tr r="M16" s="5"/>

</xml_diff>

<commit_message>
WIP: Added Blotter DB queries, Excel data provider, and initial Matrix loop
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Archana\eclipse-workspace\delta1-automation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D74CDE-0F31-433C-B311-D89CF5B1FF92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AD8014B-F10A-4EA3-B968-9500E9408777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" firstSheet="1" activeTab="1" xr2:uid="{5F4CC7F0-8BD6-41FD-85C1-DCF17C64A46A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" activeTab="2" xr2:uid="{5F4CC7F0-8BD6-41FD-85C1-DCF17C64A46A}"/>
   </bookViews>
   <sheets>
     <sheet name="Holidays" sheetId="13" r:id="rId1"/>
     <sheet name="AddTickers" sheetId="1" r:id="rId2"/>
-    <sheet name="Blotter Validations" sheetId="14" r:id="rId3"/>
+    <sheet name="BlotterValidations" sheetId="14" r:id="rId3"/>
     <sheet name="BotCommands" sheetId="2" r:id="rId4"/>
     <sheet name="TC014_DP-2260" sheetId="10" r:id="rId5"/>
     <sheet name="Import Intraday trades" sheetId="9" r:id="rId6"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="190">
   <si>
     <t>Ticker</t>
   </si>
@@ -587,9 +587,6 @@
     <t>Date</t>
   </si>
   <si>
-    <t>Expiration</t>
-  </si>
-  <si>
     <t>MSFT,INTC</t>
   </si>
   <si>
@@ -630,6 +627,26 @@
   </si>
   <si>
     <t>Run Flag</t>
+  </si>
+  <si>
+    <t>Tickers</t>
+  </si>
+  <si>
+    <t>Expirations</t>
+  </si>
+  <si>
+    <t>Mar6/Mar20</t>
+  </si>
+  <si>
+    <t>APR
+Mar/May</t>
+  </si>
+  <si>
+    <t>Apr
+Mar</t>
+  </si>
+  <si>
+    <t>Mar'25</t>
   </si>
 </sst>
 </file>
@@ -1061,80 +1078,80 @@
   <volType type="realTimeData">
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...3116730286</v>
+        <v>#N/A Requesting Data...4102721116</v>
         <stp/>
         <stp>BDP|14014614177385490883</stp>
         <tr r="M11" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3323881689</v>
+        <v>#N/A Requesting Data...4200943786</v>
         <stp/>
         <stp>BDP|17914771070757396967</stp>
         <tr r="M23" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1831997750</v>
+        <v>#N/A Requesting Data...2523175019</v>
         <stp/>
         <stp>BDP|12191885856176020024</stp>
         <tr r="M19" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3539005372</v>
+        <v>#N/A Requesting Data...4026482984</v>
         <stp/>
         <stp>BDP|11222918239606141336</stp>
         <tr r="M10" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1921182470</v>
+        <v>#N/A Requesting Data...3334715772</v>
         <stp/>
         <stp>BDP|10651803860804892507</stp>
         <tr r="M20" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2863434980</v>
+        <v>#N/A Requesting Data...4247554339</v>
         <stp/>
         <stp>BDP|11138132499892845425</stp>
         <tr r="B6" s="4"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2809252556</v>
+        <v>#N/A Requesting Data...3479047769</v>
         <stp/>
         <stp>BDP|14818210720281309974</stp>
         <tr r="F4" s="4"/>
         <tr r="M24" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3915597306</v>
+        <v>#N/A Requesting Data...3481003590</v>
         <stp/>
         <stp>BDP|17354182839553220513</stp>
         <tr r="M18" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2702786370</v>
+        <v>#N/A Requesting Data...2961707860</v>
         <stp/>
         <stp>BDP|15833637773500916777</stp>
         <tr r="M22" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3858587456</v>
+        <v>#N/A Requesting Data...3116270412</v>
         <stp/>
         <stp>BDP|10553485173797766561</stp>
         <tr r="M17" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2028483817</v>
+        <v>#N/A Requesting Data...3772991957</v>
         <stp/>
         <stp>BDP|10725320790729783234</stp>
         <tr r="M8" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2905634664</v>
+        <v>#N/A Requesting Data...3498445539</v>
         <stp/>
         <stp>BDP|15290075098549931204</stp>
         <tr r="M2" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1818396705</v>
+        <v>#N/A Requesting Data...3630203178</v>
         <stp/>
         <stp>BDP|11090127615376453378</stp>
         <tr r="M13" s="5"/>
@@ -1142,19 +1159,19 @@
     </main>
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...2463032671</v>
+        <v>#N/A Requesting Data...3760933913</v>
         <stp/>
         <stp>BDP|4236539151683226891</stp>
         <tr r="M21" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3415227157</v>
+        <v>#N/A Requesting Data...4277886170</v>
         <stp/>
         <stp>BDP|2613081399981359290</stp>
         <tr r="M12" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2945205562</v>
+        <v>#N/A Requesting Data...2989371238</v>
         <stp/>
         <stp>BDP|2154512199383777756</stp>
         <tr r="M6" s="5"/>
@@ -1172,7 +1189,7 @@
         <tr r="N23" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4254932893</v>
+        <v>#N/A Requesting Data...4075602171</v>
         <stp/>
         <stp>BDP|2219595241806083194</stp>
         <tr r="M15" s="5"/>
@@ -1185,37 +1202,37 @@
         <tr r="E16" s="4"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3813285549</v>
+        <v>#N/A Requesting Data...3421479459</v>
         <stp/>
         <stp>BDP|7276645360862777315</stp>
         <tr r="M5" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3271659411</v>
+        <v>#N/A Requesting Data...2591271917</v>
         <stp/>
         <stp>BDP|1614643148556376256</stp>
         <tr r="M9" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3800748930</v>
+        <v>#N/A Requesting Data...4290396496</v>
         <stp/>
         <stp>BDP|8389300253224362856</stp>
         <tr r="M4" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3710702205</v>
+        <v>#N/A Requesting Data...3604426337</v>
         <stp/>
         <stp>BDP|1386483162619383929</stp>
         <tr r="M3" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2644152884</v>
+        <v>#N/A Requesting Data...3084482444</v>
         <stp/>
         <stp>BDP|722161999546011081</stp>
         <tr r="M14" s="5"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2559657153</v>
+        <v>#N/A Requesting Data...3281902747</v>
         <stp/>
         <stp>BDP|281963796682346956</stp>
         <tr r="M16" s="5"/>
@@ -8013,7 +8030,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B1" t="s">
         <v>11</v>
@@ -8096,7 +8113,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -8139,7 +8156,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -8147,7 +8164,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -8155,7 +8172,7 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -8163,7 +8180,7 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -8171,7 +8188,7 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -8179,7 +8196,7 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -8187,7 +8204,7 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -8195,7 +8212,7 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -8205,21 +8222,22 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3366916-357D-497F-A92B-E1F6043DE334}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1" t="s">
         <v>184</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
       <c r="C1" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -8235,7 +8253,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -8243,7 +8261,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -8251,7 +8269,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
@@ -8259,7 +8277,42 @@
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -8280,7 +8333,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -8379,7 +8432,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -8452,7 +8505,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B1" s="77" t="s">
         <v>2</v>
@@ -8678,7 +8731,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -8859,7 +8912,7 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -9675,7 +9728,7 @@
       </c>
       <c r="N23">
         <f>IF(M23="USD",1,_xll.BDP(M23&amp;" Curncy", "PX_LAST"))</f>
-        <v>1.3586</v>
+        <v>1.3717999999999999</v>
       </c>
       <c r="P23" s="24"/>
       <c r="Q23" s="24"/>

</xml_diff>